<commit_message>
autopilot: update master + outputs + status
</commit_message>
<xml_diff>
--- a/K線西遊記/kline-btc/master/BTCUSDT_1d_1000.xlsx
+++ b/K線西遊記/kline-btc/master/BTCUSDT_1d_1000.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F1001"/>
+  <dimension ref="A1:F1079"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -22448,16 +22448,1732 @@
         <v>86670.36</v>
       </c>
       <c r="C1001" t="n">
-        <v>87973.11</v>
+        <v>88860</v>
       </c>
       <c r="D1001" t="n">
         <v>86509.63</v>
       </c>
       <c r="E1001" t="n">
-        <v>87847.07000000001</v>
+        <v>88347.08</v>
       </c>
       <c r="F1001" t="n">
-        <v>5652.86539</v>
+        <v>17766.51453</v>
+      </c>
+    </row>
+    <row r="1002">
+      <c r="A1002" t="inlineStr">
+        <is>
+          <t>2026-01-27</t>
+        </is>
+      </c>
+      <c r="B1002" t="n">
+        <v>88347.08</v>
+      </c>
+      <c r="C1002" t="n">
+        <v>89523.16</v>
+      </c>
+      <c r="D1002" t="n">
+        <v>87304.33</v>
+      </c>
+      <c r="E1002" t="n">
+        <v>89250</v>
+      </c>
+      <c r="F1002" t="n">
+        <v>13125.40425</v>
+      </c>
+    </row>
+    <row r="1003">
+      <c r="A1003" t="inlineStr">
+        <is>
+          <t>2026-01-28</t>
+        </is>
+      </c>
+      <c r="B1003" t="n">
+        <v>89249.99000000001</v>
+      </c>
+      <c r="C1003" t="n">
+        <v>90600</v>
+      </c>
+      <c r="D1003" t="n">
+        <v>88833.64999999999</v>
+      </c>
+      <c r="E1003" t="n">
+        <v>89299.99000000001</v>
+      </c>
+      <c r="F1003" t="n">
+        <v>14332.18502</v>
+      </c>
+    </row>
+    <row r="1004">
+      <c r="A1004" t="inlineStr">
+        <is>
+          <t>2026-01-29</t>
+        </is>
+      </c>
+      <c r="B1004" t="n">
+        <v>89300</v>
+      </c>
+      <c r="C1004" t="n">
+        <v>89348</v>
+      </c>
+      <c r="D1004" t="n">
+        <v>83383.33</v>
+      </c>
+      <c r="E1004" t="n">
+        <v>84650.16</v>
+      </c>
+      <c r="F1004" t="n">
+        <v>30431.38201</v>
+      </c>
+    </row>
+    <row r="1005">
+      <c r="A1005" t="inlineStr">
+        <is>
+          <t>2026-01-30</t>
+        </is>
+      </c>
+      <c r="B1005" t="n">
+        <v>84650.16</v>
+      </c>
+      <c r="C1005" t="n">
+        <v>84735.75</v>
+      </c>
+      <c r="D1005" t="n">
+        <v>81118</v>
+      </c>
+      <c r="E1005" t="n">
+        <v>84260.49000000001</v>
+      </c>
+      <c r="F1005" t="n">
+        <v>35195.84793</v>
+      </c>
+    </row>
+    <row r="1006">
+      <c r="A1006" t="inlineStr">
+        <is>
+          <t>2026-01-31</t>
+        </is>
+      </c>
+      <c r="B1006" t="n">
+        <v>84260.5</v>
+      </c>
+      <c r="C1006" t="n">
+        <v>84270.02</v>
+      </c>
+      <c r="D1006" t="n">
+        <v>75719.89999999999</v>
+      </c>
+      <c r="E1006" t="n">
+        <v>78741.09</v>
+      </c>
+      <c r="F1006" t="n">
+        <v>39491.89133</v>
+      </c>
+    </row>
+    <row r="1007">
+      <c r="A1007" t="inlineStr">
+        <is>
+          <t>2026-02-01</t>
+        </is>
+      </c>
+      <c r="B1007" t="n">
+        <v>78741.10000000001</v>
+      </c>
+      <c r="C1007" t="n">
+        <v>79424</v>
+      </c>
+      <c r="D1007" t="n">
+        <v>75700</v>
+      </c>
+      <c r="E1007" t="n">
+        <v>76968.21000000001</v>
+      </c>
+      <c r="F1007" t="n">
+        <v>25395.48168</v>
+      </c>
+    </row>
+    <row r="1008">
+      <c r="A1008" t="inlineStr">
+        <is>
+          <t>2026-02-02</t>
+        </is>
+      </c>
+      <c r="B1008" t="n">
+        <v>76968.22</v>
+      </c>
+      <c r="C1008" t="n">
+        <v>79360</v>
+      </c>
+      <c r="D1008" t="n">
+        <v>74604</v>
+      </c>
+      <c r="E1008" t="n">
+        <v>78738.61</v>
+      </c>
+      <c r="F1008" t="n">
+        <v>42273.59016</v>
+      </c>
+    </row>
+    <row r="1009">
+      <c r="A1009" t="inlineStr">
+        <is>
+          <t>2026-02-03</t>
+        </is>
+      </c>
+      <c r="B1009" t="n">
+        <v>78738.60000000001</v>
+      </c>
+      <c r="C1009" t="n">
+        <v>79186.81</v>
+      </c>
+      <c r="D1009" t="n">
+        <v>72945.5</v>
+      </c>
+      <c r="E1009" t="n">
+        <v>75770.21000000001</v>
+      </c>
+      <c r="F1009" t="n">
+        <v>39120.10889</v>
+      </c>
+    </row>
+    <row r="1010">
+      <c r="A1010" t="inlineStr">
+        <is>
+          <t>2026-02-04</t>
+        </is>
+      </c>
+      <c r="B1010" t="n">
+        <v>75770.21000000001</v>
+      </c>
+      <c r="C1010" t="n">
+        <v>76971.52</v>
+      </c>
+      <c r="D1010" t="n">
+        <v>71888</v>
+      </c>
+      <c r="E1010" t="n">
+        <v>73165.83</v>
+      </c>
+      <c r="F1010" t="n">
+        <v>38375.36</v>
+      </c>
+    </row>
+    <row r="1011">
+      <c r="A1011" t="inlineStr">
+        <is>
+          <t>2026-02-05</t>
+        </is>
+      </c>
+      <c r="B1011" t="n">
+        <v>73165.84</v>
+      </c>
+      <c r="C1011" t="n">
+        <v>73341.17999999999</v>
+      </c>
+      <c r="D1011" t="n">
+        <v>62345</v>
+      </c>
+      <c r="E1011" t="n">
+        <v>62909.86</v>
+      </c>
+      <c r="F1011" t="n">
+        <v>106298.82899</v>
+      </c>
+    </row>
+    <row r="1012">
+      <c r="A1012" t="inlineStr">
+        <is>
+          <t>2026-02-06</t>
+        </is>
+      </c>
+      <c r="B1012" t="n">
+        <v>62909.87</v>
+      </c>
+      <c r="C1012" t="n">
+        <v>71751.33</v>
+      </c>
+      <c r="D1012" t="n">
+        <v>60000</v>
+      </c>
+      <c r="E1012" t="n">
+        <v>70580.25999999999</v>
+      </c>
+      <c r="F1012" t="n">
+        <v>92539.21531</v>
+      </c>
+    </row>
+    <row r="1013">
+      <c r="A1013" t="inlineStr">
+        <is>
+          <t>2026-02-07</t>
+        </is>
+      </c>
+      <c r="B1013" t="n">
+        <v>70580.25999999999</v>
+      </c>
+      <c r="C1013" t="n">
+        <v>71690.07000000001</v>
+      </c>
+      <c r="D1013" t="n">
+        <v>67300</v>
+      </c>
+      <c r="E1013" t="n">
+        <v>69289.38</v>
+      </c>
+      <c r="F1013" t="n">
+        <v>44255.48036</v>
+      </c>
+    </row>
+    <row r="1014">
+      <c r="A1014" t="inlineStr">
+        <is>
+          <t>2026-02-08</t>
+        </is>
+      </c>
+      <c r="B1014" t="n">
+        <v>69289.37</v>
+      </c>
+      <c r="C1014" t="n">
+        <v>72271.41</v>
+      </c>
+      <c r="D1014" t="n">
+        <v>68888</v>
+      </c>
+      <c r="E1014" t="n">
+        <v>70330.38</v>
+      </c>
+      <c r="F1014" t="n">
+        <v>21420.53168</v>
+      </c>
+    </row>
+    <row r="1015">
+      <c r="A1015" t="inlineStr">
+        <is>
+          <t>2026-02-09</t>
+        </is>
+      </c>
+      <c r="B1015" t="n">
+        <v>70330.38</v>
+      </c>
+      <c r="C1015" t="n">
+        <v>71453.53</v>
+      </c>
+      <c r="D1015" t="n">
+        <v>68308</v>
+      </c>
+      <c r="E1015" t="n">
+        <v>70138</v>
+      </c>
+      <c r="F1015" t="n">
+        <v>29152.72842</v>
+      </c>
+    </row>
+    <row r="1016">
+      <c r="A1016" t="inlineStr">
+        <is>
+          <t>2026-02-10</t>
+        </is>
+      </c>
+      <c r="B1016" t="n">
+        <v>70138</v>
+      </c>
+      <c r="C1016" t="n">
+        <v>70527.59</v>
+      </c>
+      <c r="D1016" t="n">
+        <v>67800</v>
+      </c>
+      <c r="E1016" t="n">
+        <v>68841.28999999999</v>
+      </c>
+      <c r="F1016" t="n">
+        <v>20373.77072</v>
+      </c>
+    </row>
+    <row r="1017">
+      <c r="A1017" t="inlineStr">
+        <is>
+          <t>2026-02-11</t>
+        </is>
+      </c>
+      <c r="B1017" t="n">
+        <v>68841.28</v>
+      </c>
+      <c r="C1017" t="n">
+        <v>69292.88</v>
+      </c>
+      <c r="D1017" t="n">
+        <v>65756</v>
+      </c>
+      <c r="E1017" t="n">
+        <v>67082.52</v>
+      </c>
+      <c r="F1017" t="n">
+        <v>28718.24602</v>
+      </c>
+    </row>
+    <row r="1018">
+      <c r="A1018" t="inlineStr">
+        <is>
+          <t>2026-02-12</t>
+        </is>
+      </c>
+      <c r="B1018" t="n">
+        <v>67082.52</v>
+      </c>
+      <c r="C1018" t="n">
+        <v>68410.52</v>
+      </c>
+      <c r="D1018" t="n">
+        <v>65118</v>
+      </c>
+      <c r="E1018" t="n">
+        <v>66272.17</v>
+      </c>
+      <c r="F1018" t="n">
+        <v>24271.74283</v>
+      </c>
+    </row>
+    <row r="1019">
+      <c r="A1019" t="inlineStr">
+        <is>
+          <t>2026-02-13</t>
+        </is>
+      </c>
+      <c r="B1019" t="n">
+        <v>66272.17</v>
+      </c>
+      <c r="C1019" t="n">
+        <v>69482.97</v>
+      </c>
+      <c r="D1019" t="n">
+        <v>65872.46000000001</v>
+      </c>
+      <c r="E1019" t="n">
+        <v>68853.96000000001</v>
+      </c>
+      <c r="F1019" t="n">
+        <v>20244.54955</v>
+      </c>
+    </row>
+    <row r="1020">
+      <c r="A1020" t="inlineStr">
+        <is>
+          <t>2026-02-14</t>
+        </is>
+      </c>
+      <c r="B1020" t="n">
+        <v>68853.97</v>
+      </c>
+      <c r="C1020" t="n">
+        <v>70560.00999999999</v>
+      </c>
+      <c r="D1020" t="n">
+        <v>68730.13</v>
+      </c>
+      <c r="E1020" t="n">
+        <v>69822.95</v>
+      </c>
+      <c r="F1020" t="n">
+        <v>18114.78393</v>
+      </c>
+    </row>
+    <row r="1021">
+      <c r="A1021" t="inlineStr">
+        <is>
+          <t>2026-02-15</t>
+        </is>
+      </c>
+      <c r="B1021" t="n">
+        <v>69822.94</v>
+      </c>
+      <c r="C1021" t="n">
+        <v>70983</v>
+      </c>
+      <c r="D1021" t="n">
+        <v>68000</v>
+      </c>
+      <c r="E1021" t="n">
+        <v>68832.58</v>
+      </c>
+      <c r="F1021" t="n">
+        <v>22290.05208</v>
+      </c>
+    </row>
+    <row r="1022">
+      <c r="A1022" t="inlineStr">
+        <is>
+          <t>2026-02-16</t>
+        </is>
+      </c>
+      <c r="B1022" t="n">
+        <v>68832.59</v>
+      </c>
+      <c r="C1022" t="n">
+        <v>70126.67</v>
+      </c>
+      <c r="D1022" t="n">
+        <v>67294.11</v>
+      </c>
+      <c r="E1022" t="n">
+        <v>68892.42999999999</v>
+      </c>
+      <c r="F1022" t="n">
+        <v>15515.76534</v>
+      </c>
+    </row>
+    <row r="1023">
+      <c r="A1023" t="inlineStr">
+        <is>
+          <t>2026-02-17</t>
+        </is>
+      </c>
+      <c r="B1023" t="n">
+        <v>68892.42999999999</v>
+      </c>
+      <c r="C1023" t="n">
+        <v>69241.5</v>
+      </c>
+      <c r="D1023" t="n">
+        <v>66621.06</v>
+      </c>
+      <c r="E1023" t="n">
+        <v>67503.52</v>
+      </c>
+      <c r="F1023" t="n">
+        <v>16489.06921</v>
+      </c>
+    </row>
+    <row r="1024">
+      <c r="A1024" t="inlineStr">
+        <is>
+          <t>2026-02-18</t>
+        </is>
+      </c>
+      <c r="B1024" t="n">
+        <v>67503.52</v>
+      </c>
+      <c r="C1024" t="n">
+        <v>68476.22</v>
+      </c>
+      <c r="D1024" t="n">
+        <v>65870</v>
+      </c>
+      <c r="E1024" t="n">
+        <v>66461</v>
+      </c>
+      <c r="F1024" t="n">
+        <v>15492.43839</v>
+      </c>
+    </row>
+    <row r="1025">
+      <c r="A1025" t="inlineStr">
+        <is>
+          <t>2026-02-19</t>
+        </is>
+      </c>
+      <c r="B1025" t="n">
+        <v>66461</v>
+      </c>
+      <c r="C1025" t="n">
+        <v>67320</v>
+      </c>
+      <c r="D1025" t="n">
+        <v>65631.83</v>
+      </c>
+      <c r="E1025" t="n">
+        <v>67003.73</v>
+      </c>
+      <c r="F1025" t="n">
+        <v>14542.26988</v>
+      </c>
+    </row>
+    <row r="1026">
+      <c r="A1026" t="inlineStr">
+        <is>
+          <t>2026-02-20</t>
+        </is>
+      </c>
+      <c r="B1026" t="n">
+        <v>67003.73</v>
+      </c>
+      <c r="C1026" t="n">
+        <v>68318.39</v>
+      </c>
+      <c r="D1026" t="n">
+        <v>66280.2</v>
+      </c>
+      <c r="E1026" t="n">
+        <v>68020.00999999999</v>
+      </c>
+      <c r="F1026" t="n">
+        <v>35351.87091</v>
+      </c>
+    </row>
+    <row r="1027">
+      <c r="A1027" t="inlineStr">
+        <is>
+          <t>2026-02-21</t>
+        </is>
+      </c>
+      <c r="B1027" t="n">
+        <v>68020</v>
+      </c>
+      <c r="C1027" t="n">
+        <v>68698.7</v>
+      </c>
+      <c r="D1027" t="n">
+        <v>67534.69</v>
+      </c>
+      <c r="E1027" t="n">
+        <v>67975.92999999999</v>
+      </c>
+      <c r="F1027" t="n">
+        <v>8032.84131</v>
+      </c>
+    </row>
+    <row r="1028">
+      <c r="A1028" t="inlineStr">
+        <is>
+          <t>2026-02-22</t>
+        </is>
+      </c>
+      <c r="B1028" t="n">
+        <v>67975.92999999999</v>
+      </c>
+      <c r="C1028" t="n">
+        <v>68245</v>
+      </c>
+      <c r="D1028" t="n">
+        <v>67190</v>
+      </c>
+      <c r="E1028" t="n">
+        <v>67643.39999999999</v>
+      </c>
+      <c r="F1028" t="n">
+        <v>8175.13484</v>
+      </c>
+    </row>
+    <row r="1029">
+      <c r="A1029" t="inlineStr">
+        <is>
+          <t>2026-02-23</t>
+        </is>
+      </c>
+      <c r="B1029" t="n">
+        <v>67643.39</v>
+      </c>
+      <c r="C1029" t="n">
+        <v>67684.86</v>
+      </c>
+      <c r="D1029" t="n">
+        <v>63888.79</v>
+      </c>
+      <c r="E1029" t="n">
+        <v>64656.02</v>
+      </c>
+      <c r="F1029" t="n">
+        <v>33075.90923</v>
+      </c>
+    </row>
+    <row r="1030">
+      <c r="A1030" t="inlineStr">
+        <is>
+          <t>2026-02-24</t>
+        </is>
+      </c>
+      <c r="B1030" t="n">
+        <v>64656.01</v>
+      </c>
+      <c r="C1030" t="n">
+        <v>65026.75</v>
+      </c>
+      <c r="D1030" t="n">
+        <v>62510.28</v>
+      </c>
+      <c r="E1030" t="n">
+        <v>64058.15</v>
+      </c>
+      <c r="F1030" t="n">
+        <v>23102.83622</v>
+      </c>
+    </row>
+    <row r="1031">
+      <c r="A1031" t="inlineStr">
+        <is>
+          <t>2026-02-25</t>
+        </is>
+      </c>
+      <c r="B1031" t="n">
+        <v>64058.15</v>
+      </c>
+      <c r="C1031" t="n">
+        <v>69988.83</v>
+      </c>
+      <c r="D1031" t="n">
+        <v>63913.27</v>
+      </c>
+      <c r="E1031" t="n">
+        <v>67988.03999999999</v>
+      </c>
+      <c r="F1031" t="n">
+        <v>30749.99259</v>
+      </c>
+    </row>
+    <row r="1032">
+      <c r="A1032" t="inlineStr">
+        <is>
+          <t>2026-02-26</t>
+        </is>
+      </c>
+      <c r="B1032" t="n">
+        <v>67988.03999999999</v>
+      </c>
+      <c r="C1032" t="n">
+        <v>68860</v>
+      </c>
+      <c r="D1032" t="n">
+        <v>66500</v>
+      </c>
+      <c r="E1032" t="n">
+        <v>67485.17999999999</v>
+      </c>
+      <c r="F1032" t="n">
+        <v>20737.77792</v>
+      </c>
+    </row>
+    <row r="1033">
+      <c r="A1033" t="inlineStr">
+        <is>
+          <t>2026-02-27</t>
+        </is>
+      </c>
+      <c r="B1033" t="n">
+        <v>67485.19</v>
+      </c>
+      <c r="C1033" t="n">
+        <v>68216.8</v>
+      </c>
+      <c r="D1033" t="n">
+        <v>64914.46</v>
+      </c>
+      <c r="E1033" t="n">
+        <v>65872.10000000001</v>
+      </c>
+      <c r="F1033" t="n">
+        <v>21228.58424</v>
+      </c>
+    </row>
+    <row r="1034">
+      <c r="A1034" t="inlineStr">
+        <is>
+          <t>2026-02-28</t>
+        </is>
+      </c>
+      <c r="B1034" t="n">
+        <v>65872.09</v>
+      </c>
+      <c r="C1034" t="n">
+        <v>67760</v>
+      </c>
+      <c r="D1034" t="n">
+        <v>63030</v>
+      </c>
+      <c r="E1034" t="n">
+        <v>66973.25999999999</v>
+      </c>
+      <c r="F1034" t="n">
+        <v>22548.71649</v>
+      </c>
+    </row>
+    <row r="1035">
+      <c r="A1035" t="inlineStr">
+        <is>
+          <t>2026-03-01</t>
+        </is>
+      </c>
+      <c r="B1035" t="n">
+        <v>66973.25999999999</v>
+      </c>
+      <c r="C1035" t="n">
+        <v>68199.99000000001</v>
+      </c>
+      <c r="D1035" t="n">
+        <v>65056</v>
+      </c>
+      <c r="E1035" t="n">
+        <v>65776.47</v>
+      </c>
+      <c r="F1035" t="n">
+        <v>23201.85859</v>
+      </c>
+    </row>
+    <row r="1036">
+      <c r="A1036" t="inlineStr">
+        <is>
+          <t>2026-03-02</t>
+        </is>
+      </c>
+      <c r="B1036" t="n">
+        <v>65776.48</v>
+      </c>
+      <c r="C1036" t="n">
+        <v>70096</v>
+      </c>
+      <c r="D1036" t="n">
+        <v>65259.21</v>
+      </c>
+      <c r="E1036" t="n">
+        <v>68830.06</v>
+      </c>
+      <c r="F1036" t="n">
+        <v>32010.38431</v>
+      </c>
+    </row>
+    <row r="1037">
+      <c r="A1037" t="inlineStr">
+        <is>
+          <t>2026-03-03</t>
+        </is>
+      </c>
+      <c r="B1037" t="n">
+        <v>68830.06</v>
+      </c>
+      <c r="C1037" t="n">
+        <v>69258.08</v>
+      </c>
+      <c r="D1037" t="n">
+        <v>66158</v>
+      </c>
+      <c r="E1037" t="n">
+        <v>68338</v>
+      </c>
+      <c r="F1037" t="n">
+        <v>24972.2418</v>
+      </c>
+    </row>
+    <row r="1038">
+      <c r="A1038" t="inlineStr">
+        <is>
+          <t>2026-03-04</t>
+        </is>
+      </c>
+      <c r="B1038" t="n">
+        <v>68338.00999999999</v>
+      </c>
+      <c r="C1038" t="n">
+        <v>74050</v>
+      </c>
+      <c r="D1038" t="n">
+        <v>67400</v>
+      </c>
+      <c r="E1038" t="n">
+        <v>72666.77</v>
+      </c>
+      <c r="F1038" t="n">
+        <v>44919.0761</v>
+      </c>
+    </row>
+    <row r="1039">
+      <c r="A1039" t="inlineStr">
+        <is>
+          <t>2026-03-05</t>
+        </is>
+      </c>
+      <c r="B1039" t="n">
+        <v>72666.77</v>
+      </c>
+      <c r="C1039" t="n">
+        <v>73558.14999999999</v>
+      </c>
+      <c r="D1039" t="n">
+        <v>70645.47</v>
+      </c>
+      <c r="E1039" t="n">
+        <v>70890.72</v>
+      </c>
+      <c r="F1039" t="n">
+        <v>26590.51253</v>
+      </c>
+    </row>
+    <row r="1040">
+      <c r="A1040" t="inlineStr">
+        <is>
+          <t>2026-03-06</t>
+        </is>
+      </c>
+      <c r="B1040" t="n">
+        <v>70891.02</v>
+      </c>
+      <c r="C1040" t="n">
+        <v>71419.98</v>
+      </c>
+      <c r="D1040" t="n">
+        <v>67744.78</v>
+      </c>
+      <c r="E1040" t="n">
+        <v>68114.02</v>
+      </c>
+      <c r="F1040" t="n">
+        <v>22629.88722</v>
+      </c>
+    </row>
+    <row r="1041">
+      <c r="A1041" t="inlineStr">
+        <is>
+          <t>2026-03-07</t>
+        </is>
+      </c>
+      <c r="B1041" t="n">
+        <v>68114.02</v>
+      </c>
+      <c r="C1041" t="n">
+        <v>68551.03999999999</v>
+      </c>
+      <c r="D1041" t="n">
+        <v>66915.25999999999</v>
+      </c>
+      <c r="E1041" t="n">
+        <v>67262.91</v>
+      </c>
+      <c r="F1041" t="n">
+        <v>12719.54315</v>
+      </c>
+    </row>
+    <row r="1042">
+      <c r="A1042" t="inlineStr">
+        <is>
+          <t>2026-03-08</t>
+        </is>
+      </c>
+      <c r="B1042" t="n">
+        <v>67262.91</v>
+      </c>
+      <c r="C1042" t="n">
+        <v>68200</v>
+      </c>
+      <c r="D1042" t="n">
+        <v>65618.49000000001</v>
+      </c>
+      <c r="E1042" t="n">
+        <v>65971.2</v>
+      </c>
+      <c r="F1042" t="n">
+        <v>21593.63901</v>
+      </c>
+    </row>
+    <row r="1043">
+      <c r="A1043" t="inlineStr">
+        <is>
+          <t>2026-03-09</t>
+        </is>
+      </c>
+      <c r="B1043" t="n">
+        <v>65971.2</v>
+      </c>
+      <c r="C1043" t="n">
+        <v>69516.64999999999</v>
+      </c>
+      <c r="D1043" t="n">
+        <v>65821.97</v>
+      </c>
+      <c r="E1043" t="n">
+        <v>68432.16</v>
+      </c>
+      <c r="F1043" t="n">
+        <v>28896.7213</v>
+      </c>
+    </row>
+    <row r="1044">
+      <c r="A1044" t="inlineStr">
+        <is>
+          <t>2026-03-10</t>
+        </is>
+      </c>
+      <c r="B1044" t="n">
+        <v>68432.16</v>
+      </c>
+      <c r="C1044" t="n">
+        <v>71777</v>
+      </c>
+      <c r="D1044" t="n">
+        <v>68391.41</v>
+      </c>
+      <c r="E1044" t="n">
+        <v>69948.63</v>
+      </c>
+      <c r="F1044" t="n">
+        <v>32602.57726</v>
+      </c>
+    </row>
+    <row r="1045">
+      <c r="A1045" t="inlineStr">
+        <is>
+          <t>2026-03-11</t>
+        </is>
+      </c>
+      <c r="B1045" t="n">
+        <v>69948.64</v>
+      </c>
+      <c r="C1045" t="n">
+        <v>71321</v>
+      </c>
+      <c r="D1045" t="n">
+        <v>68977.91</v>
+      </c>
+      <c r="E1045" t="n">
+        <v>70191.86</v>
+      </c>
+      <c r="F1045" t="n">
+        <v>27249.27542</v>
+      </c>
+    </row>
+    <row r="1046">
+      <c r="A1046" t="inlineStr">
+        <is>
+          <t>2026-03-12</t>
+        </is>
+      </c>
+      <c r="B1046" t="n">
+        <v>70191.86</v>
+      </c>
+      <c r="C1046" t="n">
+        <v>70800</v>
+      </c>
+      <c r="D1046" t="n">
+        <v>69205.91</v>
+      </c>
+      <c r="E1046" t="n">
+        <v>70541.34</v>
+      </c>
+      <c r="F1046" t="n">
+        <v>21997.1605</v>
+      </c>
+    </row>
+    <row r="1047">
+      <c r="A1047" t="inlineStr">
+        <is>
+          <t>2026-03-13</t>
+        </is>
+      </c>
+      <c r="B1047" t="n">
+        <v>70541.34</v>
+      </c>
+      <c r="C1047" t="n">
+        <v>73913.74000000001</v>
+      </c>
+      <c r="D1047" t="n">
+        <v>70386.00999999999</v>
+      </c>
+      <c r="E1047" t="n">
+        <v>70930</v>
+      </c>
+      <c r="F1047" t="n">
+        <v>35996.61678</v>
+      </c>
+    </row>
+    <row r="1048">
+      <c r="A1048" t="inlineStr">
+        <is>
+          <t>2026-03-14</t>
+        </is>
+      </c>
+      <c r="B1048" t="n">
+        <v>70930.00999999999</v>
+      </c>
+      <c r="C1048" t="n">
+        <v>71307.92</v>
+      </c>
+      <c r="D1048" t="n">
+        <v>70317</v>
+      </c>
+      <c r="E1048" t="n">
+        <v>71211.95</v>
+      </c>
+      <c r="F1048" t="n">
+        <v>13017.24737</v>
+      </c>
+    </row>
+    <row r="1049">
+      <c r="A1049" t="inlineStr">
+        <is>
+          <t>2026-03-15</t>
+        </is>
+      </c>
+      <c r="B1049" t="n">
+        <v>71211.95</v>
+      </c>
+      <c r="C1049" t="n">
+        <v>73199</v>
+      </c>
+      <c r="D1049" t="n">
+        <v>70858.82000000001</v>
+      </c>
+      <c r="E1049" t="n">
+        <v>72815.24000000001</v>
+      </c>
+      <c r="F1049" t="n">
+        <v>14037.30704</v>
+      </c>
+    </row>
+    <row r="1050">
+      <c r="A1050" t="inlineStr">
+        <is>
+          <t>2026-03-16</t>
+        </is>
+      </c>
+      <c r="B1050" t="n">
+        <v>72815.25</v>
+      </c>
+      <c r="C1050" t="n">
+        <v>74909.08</v>
+      </c>
+      <c r="D1050" t="n">
+        <v>72270.41</v>
+      </c>
+      <c r="E1050" t="n">
+        <v>74884.67</v>
+      </c>
+      <c r="F1050" t="n">
+        <v>28409.53019</v>
+      </c>
+    </row>
+    <row r="1051">
+      <c r="A1051" t="inlineStr">
+        <is>
+          <t>2026-03-17</t>
+        </is>
+      </c>
+      <c r="B1051" t="n">
+        <v>74884.67</v>
+      </c>
+      <c r="C1051" t="n">
+        <v>76000</v>
+      </c>
+      <c r="D1051" t="n">
+        <v>73399.19</v>
+      </c>
+      <c r="E1051" t="n">
+        <v>73909.36</v>
+      </c>
+      <c r="F1051" t="n">
+        <v>24521.26636</v>
+      </c>
+    </row>
+    <row r="1052">
+      <c r="A1052" t="inlineStr">
+        <is>
+          <t>2026-03-18</t>
+        </is>
+      </c>
+      <c r="B1052" t="n">
+        <v>73909.37</v>
+      </c>
+      <c r="C1052" t="n">
+        <v>74672.34</v>
+      </c>
+      <c r="D1052" t="n">
+        <v>70500</v>
+      </c>
+      <c r="E1052" t="n">
+        <v>71246.53999999999</v>
+      </c>
+      <c r="F1052" t="n">
+        <v>23392.88093</v>
+      </c>
+    </row>
+    <row r="1053">
+      <c r="A1053" t="inlineStr">
+        <is>
+          <t>2026-03-19</t>
+        </is>
+      </c>
+      <c r="B1053" t="n">
+        <v>71246.55</v>
+      </c>
+      <c r="C1053" t="n">
+        <v>71613.78999999999</v>
+      </c>
+      <c r="D1053" t="n">
+        <v>68793.35000000001</v>
+      </c>
+      <c r="E1053" t="n">
+        <v>69930</v>
+      </c>
+      <c r="F1053" t="n">
+        <v>22364.81819</v>
+      </c>
+    </row>
+    <row r="1054">
+      <c r="A1054" t="inlineStr">
+        <is>
+          <t>2026-03-20</t>
+        </is>
+      </c>
+      <c r="B1054" t="n">
+        <v>69930.00999999999</v>
+      </c>
+      <c r="C1054" t="n">
+        <v>71367</v>
+      </c>
+      <c r="D1054" t="n">
+        <v>69388</v>
+      </c>
+      <c r="E1054" t="n">
+        <v>70510.73</v>
+      </c>
+      <c r="F1054" t="n">
+        <v>18121.16745</v>
+      </c>
+    </row>
+    <row r="1055">
+      <c r="A1055" t="inlineStr">
+        <is>
+          <t>2026-03-21</t>
+        </is>
+      </c>
+      <c r="B1055" t="n">
+        <v>70510.73</v>
+      </c>
+      <c r="C1055" t="n">
+        <v>71100.94</v>
+      </c>
+      <c r="D1055" t="n">
+        <v>68571.42</v>
+      </c>
+      <c r="E1055" t="n">
+        <v>68918.12</v>
+      </c>
+      <c r="F1055" t="n">
+        <v>13397.1675</v>
+      </c>
+    </row>
+    <row r="1056">
+      <c r="A1056" t="inlineStr">
+        <is>
+          <t>2026-03-22</t>
+        </is>
+      </c>
+      <c r="B1056" t="n">
+        <v>68918.12</v>
+      </c>
+      <c r="C1056" t="n">
+        <v>69588.78999999999</v>
+      </c>
+      <c r="D1056" t="n">
+        <v>67360.66</v>
+      </c>
+      <c r="E1056" t="n">
+        <v>67859</v>
+      </c>
+      <c r="F1056" t="n">
+        <v>14843.78682</v>
+      </c>
+    </row>
+    <row r="1057">
+      <c r="A1057" t="inlineStr">
+        <is>
+          <t>2026-03-23</t>
+        </is>
+      </c>
+      <c r="B1057" t="n">
+        <v>67859</v>
+      </c>
+      <c r="C1057" t="n">
+        <v>71817.09</v>
+      </c>
+      <c r="D1057" t="n">
+        <v>67445.17999999999</v>
+      </c>
+      <c r="E1057" t="n">
+        <v>70906.45</v>
+      </c>
+      <c r="F1057" t="n">
+        <v>28335.09119</v>
+      </c>
+    </row>
+    <row r="1058">
+      <c r="A1058" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="B1058" t="n">
+        <v>70906.45</v>
+      </c>
+      <c r="C1058" t="n">
+        <v>71400</v>
+      </c>
+      <c r="D1058" t="n">
+        <v>68923.07000000001</v>
+      </c>
+      <c r="E1058" t="n">
+        <v>70556.74000000001</v>
+      </c>
+      <c r="F1058" t="n">
+        <v>20702.42244</v>
+      </c>
+    </row>
+    <row r="1059">
+      <c r="A1059" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="B1059" t="n">
+        <v>70556.74000000001</v>
+      </c>
+      <c r="C1059" t="n">
+        <v>72026.09</v>
+      </c>
+      <c r="D1059" t="n">
+        <v>70408</v>
+      </c>
+      <c r="E1059" t="n">
+        <v>71336.53</v>
+      </c>
+      <c r="F1059" t="n">
+        <v>17719.50066</v>
+      </c>
+    </row>
+    <row r="1060">
+      <c r="A1060" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="B1060" t="n">
+        <v>71336.53</v>
+      </c>
+      <c r="C1060" t="n">
+        <v>71436.82000000001</v>
+      </c>
+      <c r="D1060" t="n">
+        <v>68153</v>
+      </c>
+      <c r="E1060" t="n">
+        <v>68820.31</v>
+      </c>
+      <c r="F1060" t="n">
+        <v>20820.45768</v>
+      </c>
+    </row>
+    <row r="1061">
+      <c r="A1061" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="B1061" t="n">
+        <v>68820.31</v>
+      </c>
+      <c r="C1061" t="n">
+        <v>69179.05</v>
+      </c>
+      <c r="D1061" t="n">
+        <v>65548.25</v>
+      </c>
+      <c r="E1061" t="n">
+        <v>66407.28</v>
+      </c>
+      <c r="F1061" t="n">
+        <v>28603.69557</v>
+      </c>
+    </row>
+    <row r="1062">
+      <c r="A1062" t="inlineStr">
+        <is>
+          <t>2026-03-28</t>
+        </is>
+      </c>
+      <c r="B1062" t="n">
+        <v>66407.28</v>
+      </c>
+      <c r="C1062" t="n">
+        <v>67288.94</v>
+      </c>
+      <c r="D1062" t="n">
+        <v>65932.09</v>
+      </c>
+      <c r="E1062" t="n">
+        <v>66377.03</v>
+      </c>
+      <c r="F1062" t="n">
+        <v>11462.39847</v>
+      </c>
+    </row>
+    <row r="1063">
+      <c r="A1063" t="inlineStr">
+        <is>
+          <t>2026-03-29</t>
+        </is>
+      </c>
+      <c r="B1063" t="n">
+        <v>66377.03999999999</v>
+      </c>
+      <c r="C1063" t="n">
+        <v>67130.5</v>
+      </c>
+      <c r="D1063" t="n">
+        <v>65000</v>
+      </c>
+      <c r="E1063" t="n">
+        <v>66010.92999999999</v>
+      </c>
+      <c r="F1063" t="n">
+        <v>10052.85584</v>
+      </c>
+    </row>
+    <row r="1064">
+      <c r="A1064" t="inlineStr">
+        <is>
+          <t>2026-03-30</t>
+        </is>
+      </c>
+      <c r="B1064" t="n">
+        <v>66010.92999999999</v>
+      </c>
+      <c r="C1064" t="n">
+        <v>68169.64999999999</v>
+      </c>
+      <c r="D1064" t="n">
+        <v>65800.59</v>
+      </c>
+      <c r="E1064" t="n">
+        <v>66797.37</v>
+      </c>
+      <c r="F1064" t="n">
+        <v>18353.38975</v>
+      </c>
+    </row>
+    <row r="1065">
+      <c r="A1065" t="inlineStr">
+        <is>
+          <t>2026-03-31</t>
+        </is>
+      </c>
+      <c r="B1065" t="n">
+        <v>66797.38</v>
+      </c>
+      <c r="C1065" t="n">
+        <v>68589.49000000001</v>
+      </c>
+      <c r="D1065" t="n">
+        <v>65998.05</v>
+      </c>
+      <c r="E1065" t="n">
+        <v>68284.48</v>
+      </c>
+      <c r="F1065" t="n">
+        <v>22105.40662</v>
+      </c>
+    </row>
+    <row r="1066">
+      <c r="A1066" t="inlineStr">
+        <is>
+          <t>2026-04-01</t>
+        </is>
+      </c>
+      <c r="B1066" t="n">
+        <v>68284.49000000001</v>
+      </c>
+      <c r="C1066" t="n">
+        <v>69310</v>
+      </c>
+      <c r="D1066" t="n">
+        <v>67578.75</v>
+      </c>
+      <c r="E1066" t="n">
+        <v>68113.92</v>
+      </c>
+      <c r="F1066" t="n">
+        <v>19020.1899</v>
+      </c>
+    </row>
+    <row r="1067">
+      <c r="A1067" t="inlineStr">
+        <is>
+          <t>2026-04-02</t>
+        </is>
+      </c>
+      <c r="B1067" t="n">
+        <v>68113.92</v>
+      </c>
+      <c r="C1067" t="n">
+        <v>68653.38</v>
+      </c>
+      <c r="D1067" t="n">
+        <v>65712.12</v>
+      </c>
+      <c r="E1067" t="n">
+        <v>66901.99000000001</v>
+      </c>
+      <c r="F1067" t="n">
+        <v>20203.47916</v>
+      </c>
+    </row>
+    <row r="1068">
+      <c r="A1068" t="inlineStr">
+        <is>
+          <t>2026-04-03</t>
+        </is>
+      </c>
+      <c r="B1068" t="n">
+        <v>66901.99000000001</v>
+      </c>
+      <c r="C1068" t="n">
+        <v>67370.42</v>
+      </c>
+      <c r="D1068" t="n">
+        <v>66282</v>
+      </c>
+      <c r="E1068" t="n">
+        <v>66964.3</v>
+      </c>
+      <c r="F1068" t="n">
+        <v>11429.13131</v>
+      </c>
+    </row>
+    <row r="1069">
+      <c r="A1069" t="inlineStr">
+        <is>
+          <t>2026-04-04</t>
+        </is>
+      </c>
+      <c r="B1069" t="n">
+        <v>66964.28999999999</v>
+      </c>
+      <c r="C1069" t="n">
+        <v>67562.92999999999</v>
+      </c>
+      <c r="D1069" t="n">
+        <v>66775.91</v>
+      </c>
+      <c r="E1069" t="n">
+        <v>67300.42</v>
+      </c>
+      <c r="F1069" t="n">
+        <v>7373.51613</v>
+      </c>
+    </row>
+    <row r="1070">
+      <c r="A1070" t="inlineStr">
+        <is>
+          <t>2026-04-05</t>
+        </is>
+      </c>
+      <c r="B1070" t="n">
+        <v>67300.42</v>
+      </c>
+      <c r="C1070" t="n">
+        <v>69136.2</v>
+      </c>
+      <c r="D1070" t="n">
+        <v>66611.66</v>
+      </c>
+      <c r="E1070" t="n">
+        <v>69034.17999999999</v>
+      </c>
+      <c r="F1070" t="n">
+        <v>11733.46752</v>
+      </c>
+    </row>
+    <row r="1071">
+      <c r="A1071" t="inlineStr">
+        <is>
+          <t>2026-04-06</t>
+        </is>
+      </c>
+      <c r="B1071" t="n">
+        <v>69034.17999999999</v>
+      </c>
+      <c r="C1071" t="n">
+        <v>70351.46000000001</v>
+      </c>
+      <c r="D1071" t="n">
+        <v>68300</v>
+      </c>
+      <c r="E1071" t="n">
+        <v>68853.66</v>
+      </c>
+      <c r="F1071" t="n">
+        <v>20281.61044</v>
+      </c>
+    </row>
+    <row r="1072">
+      <c r="A1072" t="inlineStr">
+        <is>
+          <t>2026-04-07</t>
+        </is>
+      </c>
+      <c r="B1072" t="n">
+        <v>68853.66</v>
+      </c>
+      <c r="C1072" t="n">
+        <v>72761</v>
+      </c>
+      <c r="D1072" t="n">
+        <v>67732.00999999999</v>
+      </c>
+      <c r="E1072" t="n">
+        <v>71924.22</v>
+      </c>
+      <c r="F1072" t="n">
+        <v>23750.49661</v>
+      </c>
+    </row>
+    <row r="1073">
+      <c r="A1073" t="inlineStr">
+        <is>
+          <t>2026-04-08</t>
+        </is>
+      </c>
+      <c r="B1073" t="n">
+        <v>71924.22</v>
+      </c>
+      <c r="C1073" t="n">
+        <v>72857</v>
+      </c>
+      <c r="D1073" t="n">
+        <v>70707.23</v>
+      </c>
+      <c r="E1073" t="n">
+        <v>71069.92999999999</v>
+      </c>
+      <c r="F1073" t="n">
+        <v>19802.68627</v>
+      </c>
+    </row>
+    <row r="1074">
+      <c r="A1074" t="inlineStr">
+        <is>
+          <t>2026-04-09</t>
+        </is>
+      </c>
+      <c r="B1074" t="n">
+        <v>71069.92999999999</v>
+      </c>
+      <c r="C1074" t="n">
+        <v>73145</v>
+      </c>
+      <c r="D1074" t="n">
+        <v>70466</v>
+      </c>
+      <c r="E1074" t="n">
+        <v>71787.97</v>
+      </c>
+      <c r="F1074" t="n">
+        <v>18158.42159</v>
+      </c>
+    </row>
+    <row r="1075">
+      <c r="A1075" t="inlineStr">
+        <is>
+          <t>2026-04-10</t>
+        </is>
+      </c>
+      <c r="B1075" t="n">
+        <v>71787.98</v>
+      </c>
+      <c r="C1075" t="n">
+        <v>73434</v>
+      </c>
+      <c r="D1075" t="n">
+        <v>71426.14999999999</v>
+      </c>
+      <c r="E1075" t="n">
+        <v>72962.7</v>
+      </c>
+      <c r="F1075" t="n">
+        <v>17372.63288</v>
+      </c>
+    </row>
+    <row r="1076">
+      <c r="A1076" t="inlineStr">
+        <is>
+          <t>2026-04-11</t>
+        </is>
+      </c>
+      <c r="B1076" t="n">
+        <v>72962.71000000001</v>
+      </c>
+      <c r="C1076" t="n">
+        <v>73790</v>
+      </c>
+      <c r="D1076" t="n">
+        <v>72513.09</v>
+      </c>
+      <c r="E1076" t="n">
+        <v>73043.16</v>
+      </c>
+      <c r="F1076" t="n">
+        <v>9070.943740000001</v>
+      </c>
+    </row>
+    <row r="1077">
+      <c r="A1077" t="inlineStr">
+        <is>
+          <t>2026-04-12</t>
+        </is>
+      </c>
+      <c r="B1077" t="n">
+        <v>73043.16</v>
+      </c>
+      <c r="C1077" t="n">
+        <v>73137.24000000001</v>
+      </c>
+      <c r="D1077" t="n">
+        <v>70505.88</v>
+      </c>
+      <c r="E1077" t="n">
+        <v>70740.98</v>
+      </c>
+      <c r="F1077" t="n">
+        <v>13472.46801</v>
+      </c>
+    </row>
+    <row r="1078">
+      <c r="A1078" t="inlineStr">
+        <is>
+          <t>2026-04-13</t>
+        </is>
+      </c>
+      <c r="B1078" t="n">
+        <v>70741.56</v>
+      </c>
+      <c r="C1078" t="n">
+        <v>74900</v>
+      </c>
+      <c r="D1078" t="n">
+        <v>70566.99000000001</v>
+      </c>
+      <c r="E1078" t="n">
+        <v>74417.99000000001</v>
+      </c>
+      <c r="F1078" t="n">
+        <v>24230.21625</v>
+      </c>
+    </row>
+    <row r="1079">
+      <c r="A1079" t="inlineStr">
+        <is>
+          <t>2026-04-14</t>
+        </is>
+      </c>
+      <c r="B1079" t="n">
+        <v>74418</v>
+      </c>
+      <c r="C1079" t="n">
+        <v>74489.49000000001</v>
+      </c>
+      <c r="D1079" t="n">
+        <v>74411.36</v>
+      </c>
+      <c r="E1079" t="n">
+        <v>74484.49000000001</v>
+      </c>
+      <c r="F1079" t="n">
+        <v>73.16636</v>
       </c>
     </row>
   </sheetData>

</xml_diff>